<commit_message>
Update index: 3003 → 3304 [scan complete - 9 businesses found, 23-07-2026]
Scanned addresses from index 3003 to 3303 (301 addresses).
Found 9 businesses in Jerusalem arnona database range.
Updated daily Excel report with all confirmed businesses.
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:23-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:23-07-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="דוח נכסים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="דוח נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,17 +26,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -49,38 +43,8 @@
         <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2D9F3"/>
-        <bgColor rgb="00E2D9F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1ECF1"/>
-        <bgColor rgb="00D1ECF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-        <bgColor rgb="00F8D7DA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -88,50 +52,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -498,19 +426,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -547,212 +475,248 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>ברגמן ענת</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>בית הכרם 16</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>מרפאת שיניים</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.b144.co.il/%D7%A8%D7%95%D7%A4%D7%90%D7%99-%D7%A9%D7%99%D7%A0%D7%99%D7%99%D7%9D/%D7%99%D7%A8%D7%95%D7%A9%D7%9C%D7%99%D7%9D/%D7%91%D7%99%D7%AA-%D7%94%D7%9B%D7%A8%D7%9D/</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>לזרוס מרים</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>בית הערבה 3</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>פסיכותרפיה</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80115518/40230/</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>ישיבת מדרש שמואל</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>בית וגן 52</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>ישיבה</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/33522670/20010/</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>אילת חן</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>בית וגן 25</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>ביגוד והנעלה</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>https://bayitvagan.org/business/</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="inlineStr"/>
-      <c r="G5" s="9" t="inlineStr"/>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>מיקי מתנות</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>בית וגן 74</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>חנות מתנות</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/31213570/33240/</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr"/>
-      <c r="G6" s="11" t="inlineStr"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>ברנשטיין משה</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>בית וגן 76</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>רואה חשבון</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/32002190/46140/</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>https://easy.co.il/page/25991886</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr"/>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>פרחי אטל</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>בית וגן 96</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>חנות פרחים</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80317220/40680/</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>בית חנינא - הפצה ושיווק בע"מ</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>בית חנינא החדשה 33</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>הפצה ושיווק תרופות</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.b144.co.il/b144_sip/401C041345746C5B4D170715/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>אברמוביץ אבי</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>בלפור 4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>עורכי דין</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/38168730/38010/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>גן לימור</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>אריה בן אליעזר 47</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>גני ילדים ומעונות</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80105761/10880/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>בר כל - ברכת הארץ</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>אריה בן אליעזר 47</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>סופרמרקט</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80312450/35760/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>שרביט דוד</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>אריה בן אליעזר 57</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>מורה נהיגה</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/6139920/24600/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>יוסי גינון</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>אריה בן אליעזר 43</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>שירותי גינון</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80173016/11000/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>קיסר רן</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>אריה בן אליעזר 57</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>יועץ מס</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80229732/26760/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>יאנוש גז</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>אריה בן אליעזר 65</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>שירותי גז</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80169286/9530/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>אהרון אריאל לביא</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>אריה בן אליעזר 82</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>מרצה</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80058089/32150/</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add scan results for 23-07-2026: 20 businesses found, index 3931→4809
- Excel report with 20 businesses across ברכת אברהם, ברנשטיין פרץ,
  ברניקי, גבעת שאול, גבעת קנדה, גדוד חרמש, גולומב, גלבר
- generate_excel_report.py script used to produce the formatted report
- Index updated to 4809 (scan stopped at token budget limit)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5r2S3tefJm2EzVxsSfran
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:23-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:23-07-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="דוח נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ממצאים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,11 +26,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +43,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,10 +70,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,16 +446,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,247 +496,596 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>בית חנינא - הפצה ושיווק בע"מ</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>בית חנינא החדשה 33</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>הפצה ושיווק תרופות</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://www.b144.co.il/b144_sip/401C041345746C5B4D170715/</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>יש חסד</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ברכת אברהם 22, ירושלים</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>סופרמרקטים ומכולות</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80056577/35760/</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>http://www.yesh.co.il</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>אברמוביץ אבי</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>בלפור 4</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>בית מרקחת- מאוחדת</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>ברכת אברהם 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>בתי מרקחת</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80123798/8150/</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>http://www.meuhedet.co.il</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>מחסן הבשר</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>ברכת אברהם 4, ירושלים</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>קצביות</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80012629/2490/</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>אורנג' מירה</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>ברכת אברהם 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>הריון ולידה</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80248063/14165/</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>מאוחדת</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ברכת אברהם 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>קופות חולים</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80270680/43950/</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.meuhedet.co.il/</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>בן-עמי שוקי</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ברנשטיין פרץ 22, ירושלים</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>עורכי דין</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/38168730/38010/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>גן לימור</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 47</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>גני ילדים ומעונות</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80105761/10880/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>בר כל - ברכת הארץ</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 47</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>סופרמרקט</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80312450/35760/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>שרביט דוד</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 57</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>מורה נהיגה</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/6139920/24600/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>יוסי גינון</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 43</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>שירותי גינון</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80173016/11000/</t>
-        </is>
-      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/233090/38190/</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>קיסר רן</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 57</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>יועץ מס</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80229732/26760/</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ד"ר חמו יצחק</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ברנשטיין פרץ 46, ירושלים</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>רפואת עיניים</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://d.co.il/24526470/46560</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>יאנוש גז</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 65</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>שירותי גז</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80169286/9530/</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>אוחנה מוטי</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>ברנשטיין פרץ 6, ירושלים</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>שירותים</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/25707940/14625/</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>אהרון אריאל לביא</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 82</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>מרצה</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80058089/32150/</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>סטודיו דוב אברמסון</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ברניקי 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>עיצוב גרפי</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80184921/11380/</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>סלכל בו - סלסילה</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>גבעת שאול 24, ירושלים</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>סופרמרקטים ומכולות</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/12702890/35760/</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>המלך החסיד</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>גבעת שאול 25, ירושלים</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>הדפסה דיגיטלית</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/76762080/12390/</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>פריד הנדסה בהנהלת פרידבורג חזקיהו</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>גבעת שאול 24, ירושלים</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>הנדסה ותכנון</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80140237/26270/</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>טליס - tali's</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>גבעת קנדה 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>עיצוב אריזות</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80068899/3970/</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>כהן סימה</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>גבעת קנדה 31, ירושלים</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>מורים לנהיגה</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/37797660/8450/</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>מדיה - ווייז</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>גדוד חרמש 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>מדיה ופרסום</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/7351750/40920/</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>דוד שירותי צבע</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>גדוד חרמש 16, ירושלים</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>צבעים וסיידים</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80087602/41160/</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>אפי נכסים</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>גדוד חרמש 8, ירושלים</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>מתווכים ומשרדי תיווך</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/71534970/32970/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>אברהם יואב</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>גדוד חרמש 15, ירושלים</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>חשמלאי</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/11809420/17910/</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>דלאל מוטי</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>גולומב 23, ירושלים</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>שירותי ייעוץ</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/76691530/2410/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>לויתן בני</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>גלבר 14, ירושלים</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>גישור ויישוב סכסוכים</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/71620430/9880/</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update index 4809 → 4925 [scan complete] — add business report 23-07-2026
Scanned indices 4809-4924 (גליק נלסון through גרוזנברג).
Found 7 businesses. Excel report added to 'excel outputs/'.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:23-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:23-07-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="דוח נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ממצאים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,11 +26,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -40,11 +52,25 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,14 +78,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="thin">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="thin">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,19 +484,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -475,250 +533,229 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>בית חנינא - הפצה ושיווק בע"מ</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>בית חנינא החדשה 33</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>הפצה ושיווק תרופות</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>צדוק יחיאל - שיפוצים</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>נלסון גליק 11, ירושלים</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>שיפוצים ובנייה</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://www.b144.co.il/b144_sip/401C041345746C5B4D170715/</t>
-        </is>
-      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.t.co.il/Business/Card-280502.html</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>אברמוביץ אבי</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>בלפור 4</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>עורכי דין</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>ד"ר גליק בנימין</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>נלסון גליק 27, רמות אלון ירושלים</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>רופא ילדים ✅</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/38168730/38010/</t>
-        </is>
-      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/574480/46200/</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/page/20592173</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>גן לימור</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 47</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>גני ילדים ומעונות</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>חשמל חכם</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>נלסון גליק 38, רמות אלון ירושלים</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>מוצרי חשמל ואלקטרוניקה</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80105761/10880/</t>
-        </is>
-      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80120878/17850/</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/en/page/9208951</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>בר כל - ברכת הארץ</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 47</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>סופרמרקט</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>אשר אביטן - משרד עו"ד</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>נלסון גליק 42/2, ירושלים</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>עורכי דין ✅</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80312450/35760/</t>
-        </is>
-      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.t.co.il/Business/Card-669189.html</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>שרביט דוד</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 57</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>מורה נהיגה</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>גל-יה סוכנות נכסים</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>גלעדי 8, ירושלים</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>תיווך נדל"ן</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/6139920/24600/</t>
-        </is>
-      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80073953/32970/</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>יוסי גינון</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 43</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>שירותי גינון</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>אריאל איילון</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>גלעדי 12, ירושלים</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>צלמים וסטודיו לצילום</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80173016/11000/</t>
-        </is>
-      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/41637700/42450/</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>קיסר רן</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 57</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>יועץ מס</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>מוזיאון אסירי המחתרות בירושלים</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>גרוזנברג 13, ירושלים</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>מוזיאון</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80229732/26760/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>יאנוש גז</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 65</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>שירותי גז</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80169286/9530/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>אהרון אריאל לביא</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>אריה בן אליעזר 82</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>מרצה</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80058089/32150/</t>
-        </is>
-      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/23628530/24000/</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId9"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>